<commit_message>
Update HideUnhideWU.ps1 and InstallUninstallWU.ps1 as self-contained script accepting parameters or using environment variables provided by Workspace ONE Scripts.
</commit_message>
<xml_diff>
--- a/Windows Update Ring Deferral Calculator.xlsx
+++ b/Windows Update Ring Deferral Calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/helmlingp/GitHub/apps_WindowsUpdates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27ABEFA-4C2C-9346-9735-1A0CD4F65E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6069031-C4B4-944B-9DF1-F379FF714B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{78992652-D20F-B64E-BD2A-348D49042B90}"/>
+    <workbookView xWindow="18660" yWindow="1540" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{78992652-D20F-B64E-BD2A-348D49042B90}"/>
   </bookViews>
   <sheets>
     <sheet name="Deferral Calc" sheetId="1" r:id="rId1"/>
@@ -659,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -706,19 +706,15 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -726,22 +722,22 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -750,7 +746,7 @@
     <xf numFmtId="0" fontId="7" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -775,14 +771,13 @@
     <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1303,47 +1298,47 @@
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="23"/>
       <c r="B1" s="23"/>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" ht="29">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="36" t="s">
+      <c r="F2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="37" t="s">
+      <c r="G2" s="35" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="21">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
@@ -1352,19 +1347,19 @@
       <c r="B4" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="36" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="F4" s="38" t="s">
+      <c r="F4" s="36" t="s">
         <v>114</v>
       </c>
-      <c r="G4" s="38" t="s">
+      <c r="G4" s="36" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1375,19 +1370,19 @@
       <c r="B5" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="F5" s="39" t="s">
+      <c r="F5" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="37" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1398,10 +1393,10 @@
       <c r="B6" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="37" t="s">
         <v>118</v>
       </c>
       <c r="E6" s="12"/>
@@ -1415,7 +1410,7 @@
       <c r="B7" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="36">
         <v>7</v>
       </c>
       <c r="D7" s="12"/>
@@ -1430,7 +1425,7 @@
       <c r="B8" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="36">
         <v>14</v>
       </c>
       <c r="D8" s="12"/>
@@ -1439,41 +1434,41 @@
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
     </row>
     <row r="10" spans="1:7" ht="21">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="8" t="s">
@@ -1482,7 +1477,7 @@
       <c r="B12" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="9"/>
@@ -1497,7 +1492,7 @@
       <c r="B13" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="39" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="9"/>
@@ -1512,7 +1507,7 @@
       <c r="B14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C14" s="40" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="9"/>
@@ -1527,19 +1522,19 @@
       <c r="B15" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="38">
+      <c r="C15" s="36">
         <v>0</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="36">
         <v>3</v>
       </c>
-      <c r="E15" s="38">
+      <c r="E15" s="36">
         <v>8</v>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="36">
         <v>13</v>
       </c>
-      <c r="G15" s="38">
+      <c r="G15" s="36">
         <v>18</v>
       </c>
     </row>
@@ -1561,15 +1556,15 @@
       <c r="B17" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="43" t="s">
+      <c r="C17" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="41" t="s">
         <v>119</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
-      <c r="G17" s="46" t="s">
+      <c r="G17" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1580,13 +1575,13 @@
       <c r="B18" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="42" t="s">
         <v>66</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
-      <c r="G18" s="38" t="s">
+      <c r="G18" s="36" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1597,13 +1592,13 @@
       <c r="B19" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="44" t="s">
+      <c r="C19" s="42" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
-      <c r="G19" s="47">
+      <c r="G19" s="45">
         <v>0.125</v>
       </c>
     </row>
@@ -1614,13 +1609,13 @@
       <c r="B20" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="44">
+      <c r="C20" s="42">
         <v>12</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-      <c r="G20" s="38">
+      <c r="G20" s="36">
         <v>16</v>
       </c>
     </row>
@@ -1631,13 +1626,13 @@
       <c r="B21" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C21" s="38">
+      <c r="C21" s="36">
         <v>8</v>
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
-      <c r="G21" s="38">
+      <c r="G21" s="36">
         <v>7</v>
       </c>
     </row>
@@ -1648,7 +1643,7 @@
       <c r="B22" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="38">
+      <c r="C22" s="36">
         <v>1</v>
       </c>
       <c r="D22" s="9"/>
@@ -1663,7 +1658,7 @@
       <c r="B23" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="38">
+      <c r="C23" s="36">
         <v>2</v>
       </c>
       <c r="D23" s="9"/>
@@ -1678,7 +1673,7 @@
       <c r="B24" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="44" t="s">
+      <c r="C24" s="42" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="9"/>
@@ -1693,7 +1688,7 @@
       <c r="B25" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="44" t="s">
+      <c r="C25" s="42" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="9"/>
@@ -1708,7 +1703,7 @@
       <c r="B26" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="38">
+      <c r="C26" s="36">
         <v>15</v>
       </c>
       <c r="D26" s="9"/>
@@ -1723,10 +1718,10 @@
       <c r="B27" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="38" t="s">
+      <c r="C27" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="43" t="s">
         <v>60</v>
       </c>
       <c r="E27" s="12"/>
@@ -1740,7 +1735,7 @@
       <c r="B28" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="38">
+      <c r="C28" s="36">
         <v>4</v>
       </c>
       <c r="D28" s="9"/>
@@ -1755,7 +1750,7 @@
       <c r="B29" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C29" s="38">
+      <c r="C29" s="36">
         <v>15</v>
       </c>
       <c r="D29" s="9"/>
@@ -1781,7 +1776,7 @@
       <c r="B31" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C31" s="38" t="s">
+      <c r="C31" s="36" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="9"/>
@@ -1796,7 +1791,7 @@
       <c r="B32" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="38" t="s">
+      <c r="C32" s="36" t="s">
         <v>30</v>
       </c>
       <c r="D32" s="9"/>
@@ -1811,7 +1806,7 @@
       <c r="B33" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="C33" s="38">
+      <c r="C33" s="36">
         <v>22</v>
       </c>
       <c r="D33" s="9"/>
@@ -1837,7 +1832,7 @@
       <c r="B35" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C35" s="38" t="s">
+      <c r="C35" s="36" t="s">
         <v>53</v>
       </c>
       <c r="D35" s="9"/>
@@ -1852,7 +1847,7 @@
       <c r="B36" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="38" t="s">
+      <c r="C36" s="36" t="s">
         <v>26</v>
       </c>
       <c r="D36" s="9"/>
@@ -1867,7 +1862,7 @@
       <c r="B37" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="38" t="s">
+      <c r="C37" s="36" t="s">
         <v>40</v>
       </c>
       <c r="D37" s="9"/>
@@ -1882,7 +1877,7 @@
       <c r="B38" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C38" s="38" t="s">
+      <c r="C38" s="36" t="s">
         <v>40</v>
       </c>
       <c r="D38" s="9"/>
@@ -1908,7 +1903,7 @@
       <c r="B40" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="C40" s="38" t="s">
+      <c r="C40" s="36" t="s">
         <v>66</v>
       </c>
       <c r="D40" s="8"/>
@@ -1941,22 +1936,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="4" customFormat="1" ht="42">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="F1" s="30" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1967,12 +1962,12 @@
       <c r="B2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="48">
+      <c r="C2" s="46">
         <v>2</v>
       </c>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
@@ -1981,12 +1976,12 @@
       <c r="B3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="48">
+      <c r="C3" s="46">
         <v>0</v>
       </c>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
@@ -1995,12 +1990,12 @@
       <c r="B4" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="48">
+      <c r="C4" s="46">
         <v>5</v>
       </c>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
@@ -2009,12 +2004,12 @@
       <c r="B5" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="49">
+      <c r="C5" s="38">
         <v>1</v>
       </c>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="8" t="s">
@@ -2023,12 +2018,12 @@
       <c r="B6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="49">
-        <v>600</v>
-      </c>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
+      <c r="C6" s="38">
+        <v>300</v>
+      </c>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
@@ -2037,12 +2032,12 @@
       <c r="B7" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="49">
+      <c r="C7" s="38">
         <v>60</v>
       </c>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
@@ -2051,12 +2046,9 @@
       <c r="B8" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="48">
+      <c r="C8" s="46">
         <v>64</v>
       </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
@@ -2065,12 +2057,9 @@
       <c r="B9" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="48">
+      <c r="C9" s="46">
         <v>1</v>
       </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
@@ -2079,16 +2068,16 @@
       <c r="B10" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="C10" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="50" t="s">
+      <c r="D10" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="50" t="s">
+      <c r="E10" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="50" t="s">
+      <c r="F10" s="47" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2107,9 +2096,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2324,27 +2316,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50788E35-BDCC-4343-87B0-3A4E866EE54F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C72EFAB-9C1C-419C-A030-CA7E23D2BD2D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="8e03c918-7659-4e8f-9051-23ec0b543ed8"/>
-    <ds:schemaRef ds:uri="acb0bacd-5e67-4f50-a132-1b36a8c4b0dc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2369,9 +2349,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C72EFAB-9C1C-419C-A030-CA7E23D2BD2D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50788E35-BDCC-4343-87B0-3A4E866EE54F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="8e03c918-7659-4e8f-9051-23ec0b543ed8"/>
+    <ds:schemaRef ds:uri="acb0bacd-5e67-4f50-a132-1b36a8c4b0dc"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>